<commit_message>
actualizarea cerintelor functionale, arhitecturii si testarii
</commit_message>
<xml_diff>
--- a/Cerinte_functionale.xlsx
+++ b/Cerinte_functionale.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D&amp;A\Documents\APSII_Curierat\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\danni\Desktop\Curierat_Optimizare-main\Curierat_Optimizare-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F55249E-E8F6-44AD-9D35-B0F25DE1EE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B246FAA8-FAB8-463C-8B4D-2F914872C6A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{2904E1B8-2E86-47D5-BF63-1CE4BA91B30C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{2904E1B8-2E86-47D5-BF63-1CE4BA91B30C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Nr.</t>
   </si>
@@ -156,6 +156,21 @@
   </si>
   <si>
     <t>Primire notificari</t>
+  </si>
+  <si>
+    <t>Reprogramare Livrare Colet</t>
+  </si>
+  <si>
+    <t>REQ-9</t>
+  </si>
+  <si>
+    <t>Sistemul trebuie sa permita Clientului sa modifice data de livrare.</t>
+  </si>
+  <si>
+    <t>Sistemul trebuie sa notifice Curierul in timp real cand un colet din ruta sa activa a fost reprogramat.</t>
+  </si>
+  <si>
+    <t>REQ-9.1</t>
   </si>
 </sst>
 </file>
@@ -207,10 +222,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -545,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{295664DB-52C9-4C66-B557-B859D88D5693}">
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="139" customWidth="1"/>
@@ -656,13 +671,13 @@
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="1"/>
+      <c r="B17" s="2"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -675,7 +690,7 @@
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="1" t="s">
         <v>33</v>
       </c>
     </row>
@@ -696,7 +711,7 @@
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -717,7 +732,7 @@
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -738,7 +753,7 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="1" t="s">
         <v>36</v>
       </c>
     </row>
@@ -751,7 +766,7 @@
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B37" s="2" t="s">
+      <c r="B37" s="1" t="s">
         <v>37</v>
       </c>
     </row>
@@ -772,7 +787,7 @@
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B41" s="2" t="s">
+      <c r="B41" s="1" t="s">
         <v>38</v>
       </c>
     </row>
@@ -785,7 +800,7 @@
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B44" s="2" t="s">
+      <c r="B44" s="1" t="s">
         <v>39</v>
       </c>
     </row>
@@ -795,6 +810,27 @@
       </c>
       <c r="B45" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B47" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>44</v>
+      </c>
+      <c r="B49" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>